<commit_message>
Add milestone catalog and redesign vehicle brief UI
</commit_message>
<xml_diff>
--- a/sample_lrp.xlsx
+++ b/sample_lrp.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Subhash/LaunchIQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A1C36A-2B25-C64D-8A11-DBA958F0123F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5768F99-D016-D047-BDF1-4207B58E6731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34560" yWindow="-340" windowWidth="38400" windowHeight="21000" xr2:uid="{6187741E-9FC1-9544-B488-B14C961CEA76}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$DC$293</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1857,6 +1860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B013508-E228-5F48-8A4D-5ECE74B70E01}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:DC293"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2264,7 +2268,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
         <v>83</v>
       </c>
@@ -2439,7 +2443,7 @@
       <c r="DB2" s="23"/>
       <c r="DC2" s="23"/>
     </row>
-    <row r="3" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>83</v>
       </c>
@@ -2626,7 +2630,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>83</v>
       </c>
@@ -2815,7 +2819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>83</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>83</v>
       </c>
@@ -3189,7 +3193,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>83</v>
       </c>
@@ -3354,7 +3358,7 @@
       <c r="DB7" s="23"/>
       <c r="DC7" s="23"/>
     </row>
-    <row r="8" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
         <v>83</v>
       </c>
@@ -3523,7 +3527,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="9" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -3692,7 +3696,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="10" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
         <v>83</v>
       </c>
@@ -3861,7 +3865,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
         <v>83</v>
       </c>
@@ -4030,7 +4034,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
         <v>83</v>
       </c>
@@ -4199,7 +4203,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
         <v>83</v>
       </c>
@@ -4366,7 +4370,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
         <v>83</v>
       </c>
@@ -4533,7 +4537,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
         <v>83</v>
       </c>
@@ -4700,7 +4704,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
         <v>83</v>
       </c>
@@ -4865,7 +4869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
         <v>83</v>
       </c>
@@ -5052,7 +5056,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
         <v>83</v>
       </c>
@@ -5235,7 +5239,7 @@
       </c>
       <c r="DC18" s="23"/>
     </row>
-    <row r="19" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
         <v>83</v>
       </c>
@@ -5418,7 +5422,7 @@
       </c>
       <c r="DC19" s="23"/>
     </row>
-    <row r="20" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
         <v>95</v>
       </c>
@@ -5609,7 +5613,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="21" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
         <v>95</v>
       </c>
@@ -5802,7 +5806,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
         <v>95</v>
       </c>
@@ -5995,7 +5999,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
         <v>95</v>
       </c>
@@ -6186,7 +6190,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
         <v>95</v>
       </c>
@@ -6379,7 +6383,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
         <v>95</v>
       </c>
@@ -6572,7 +6576,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
         <v>95</v>
       </c>
@@ -6759,7 +6763,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
         <v>95</v>
       </c>
@@ -6954,7 +6958,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
         <v>95</v>
       </c>
@@ -7145,7 +7149,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
         <v>95</v>
       </c>
@@ -7328,7 +7332,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
         <v>95</v>
       </c>
@@ -7521,7 +7525,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
         <v>95</v>
       </c>
@@ -7706,7 +7710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
         <v>95</v>
       </c>
@@ -7885,7 +7889,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="10" t="s">
         <v>95</v>
       </c>
@@ -8068,7 +8072,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
         <v>95</v>
       </c>
@@ -8255,7 +8259,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
         <v>95</v>
       </c>
@@ -8444,7 +8448,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="36" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="10" t="s">
         <v>95</v>
       </c>
@@ -8625,7 +8629,7 @@
       </c>
       <c r="DC36" s="23"/>
     </row>
-    <row r="37" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
         <v>95</v>
       </c>
@@ -8810,7 +8814,7 @@
       </c>
       <c r="DC37" s="23"/>
     </row>
-    <row r="38" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
         <v>95</v>
       </c>
@@ -8999,7 +9003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
         <v>95</v>
       </c>
@@ -9186,7 +9190,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
         <v>95</v>
       </c>
@@ -9377,7 +9381,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="10" t="s">
         <v>95</v>
       </c>
@@ -9566,7 +9570,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="10" t="s">
         <v>95</v>
       </c>
@@ -9753,7 +9757,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
         <v>95</v>
       </c>
@@ -9942,7 +9946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10" t="s">
         <v>95</v>
       </c>
@@ -10125,7 +10129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10" t="s">
         <v>95</v>
       </c>
@@ -10310,7 +10314,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10" t="s">
         <v>95</v>
       </c>
@@ -10499,7 +10503,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
         <v>95</v>
       </c>
@@ -10686,7 +10690,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="48" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10" t="s">
         <v>95</v>
       </c>
@@ -10875,7 +10879,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10" t="s">
         <v>95</v>
       </c>
@@ -11068,7 +11072,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10" t="s">
         <v>95</v>
       </c>
@@ -11251,7 +11255,7 @@
       </c>
       <c r="DC50" s="23"/>
     </row>
-    <row r="51" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10" t="s">
         <v>95</v>
       </c>
@@ -11428,7 +11432,7 @@
       <c r="DB51" s="23"/>
       <c r="DC51" s="23"/>
     </row>
-    <row r="52" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10" t="s">
         <v>95</v>
       </c>
@@ -11593,7 +11597,7 @@
       <c r="DB52" s="23"/>
       <c r="DC52" s="23"/>
     </row>
-    <row r="53" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10" t="s">
         <v>95</v>
       </c>
@@ -11778,7 +11782,7 @@
       </c>
       <c r="DC53" s="23"/>
     </row>
-    <row r="54" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10" t="s">
         <v>95</v>
       </c>
@@ -11963,7 +11967,7 @@
       </c>
       <c r="DC54" s="23"/>
     </row>
-    <row r="55" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10" t="s">
         <v>95</v>
       </c>
@@ -12128,7 +12132,7 @@
       <c r="DB55" s="23"/>
       <c r="DC55" s="23"/>
     </row>
-    <row r="56" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="10" t="s">
         <v>95</v>
       </c>
@@ -12293,7 +12297,7 @@
       <c r="DB56" s="23"/>
       <c r="DC56" s="23"/>
     </row>
-    <row r="57" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10" t="s">
         <v>95</v>
       </c>
@@ -12458,7 +12462,7 @@
       <c r="DB57" s="23"/>
       <c r="DC57" s="23"/>
     </row>
-    <row r="58" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="10" t="s">
         <v>95</v>
       </c>
@@ -12645,7 +12649,7 @@
       </c>
       <c r="DC58" s="23"/>
     </row>
-    <row r="59" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="10" t="s">
         <v>95</v>
       </c>
@@ -12828,7 +12832,7 @@
       <c r="DB59" s="23"/>
       <c r="DC59" s="23"/>
     </row>
-    <row r="60" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10" t="s">
         <v>95</v>
       </c>
@@ -12995,7 +12999,7 @@
       <c r="DB60" s="23"/>
       <c r="DC60" s="23"/>
     </row>
-    <row r="61" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10" t="s">
         <v>95</v>
       </c>
@@ -13156,7 +13160,7 @@
       <c r="DB61" s="23"/>
       <c r="DC61" s="23"/>
     </row>
-    <row r="62" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10" t="s">
         <v>95</v>
       </c>
@@ -13341,7 +13345,7 @@
       </c>
       <c r="DC62" s="23"/>
     </row>
-    <row r="63" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10" t="s">
         <v>95</v>
       </c>
@@ -13522,7 +13526,7 @@
       <c r="DB63" s="23"/>
       <c r="DC63" s="23"/>
     </row>
-    <row r="64" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10" t="s">
         <v>95</v>
       </c>
@@ -13687,7 +13691,7 @@
       <c r="DB64" s="23"/>
       <c r="DC64" s="23"/>
     </row>
-    <row r="65" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="10" t="s">
         <v>95</v>
       </c>
@@ -13848,7 +13852,7 @@
       <c r="DB65" s="23"/>
       <c r="DC65" s="23"/>
     </row>
-    <row r="66" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="10" t="s">
         <v>95</v>
       </c>
@@ -14033,7 +14037,7 @@
       </c>
       <c r="DC66" s="23"/>
     </row>
-    <row r="67" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="10" t="s">
         <v>95</v>
       </c>
@@ -14214,7 +14218,7 @@
       <c r="DB67" s="23"/>
       <c r="DC67" s="23"/>
     </row>
-    <row r="68" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="10" t="s">
         <v>95</v>
       </c>
@@ -14377,7 +14381,7 @@
       <c r="DB68" s="23"/>
       <c r="DC68" s="23"/>
     </row>
-    <row r="69" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="10" t="s">
         <v>95</v>
       </c>
@@ -14536,7 +14540,7 @@
       <c r="DB69" s="23"/>
       <c r="DC69" s="23"/>
     </row>
-    <row r="70" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
         <v>95</v>
       </c>
@@ -14715,7 +14719,7 @@
       </c>
       <c r="DC70" s="23"/>
     </row>
-    <row r="71" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="10" t="s">
         <v>95</v>
       </c>
@@ -14890,7 +14894,7 @@
       <c r="DB71" s="23"/>
       <c r="DC71" s="23"/>
     </row>
-    <row r="72" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="10" t="s">
         <v>95</v>
       </c>
@@ -15053,7 +15057,7 @@
       <c r="DB72" s="23"/>
       <c r="DC72" s="23"/>
     </row>
-    <row r="73" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="10" t="s">
         <v>95</v>
       </c>
@@ -15212,7 +15216,7 @@
       <c r="DB73" s="23"/>
       <c r="DC73" s="23"/>
     </row>
-    <row r="74" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="10" t="s">
         <v>95</v>
       </c>
@@ -15373,7 +15377,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="75" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="10" t="s">
         <v>95</v>
       </c>
@@ -15534,7 +15538,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="10" t="s">
         <v>95</v>
       </c>
@@ -15695,7 +15699,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="77" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="10" t="s">
         <v>95</v>
       </c>
@@ -15856,7 +15860,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="78" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="10" t="s">
         <v>95</v>
       </c>
@@ -16017,7 +16021,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="79" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="10" t="s">
         <v>104</v>
       </c>
@@ -16188,7 +16192,7 @@
         <v>2194</v>
       </c>
     </row>
-    <row r="80" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="10" t="s">
         <v>104</v>
       </c>
@@ -16359,7 +16363,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="81" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="10" t="s">
         <v>104</v>
       </c>
@@ -16530,7 +16534,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="82" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="10" t="s">
         <v>104</v>
       </c>
@@ -16701,7 +16705,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="83" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="10" t="s">
         <v>104</v>
       </c>
@@ -16870,7 +16874,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="84" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="10" t="s">
         <v>104</v>
       </c>
@@ -17059,7 +17063,7 @@
         <v>27600</v>
       </c>
     </row>
-    <row r="85" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="10" t="s">
         <v>104</v>
       </c>
@@ -17218,7 +17222,7 @@
       <c r="DB85" s="23"/>
       <c r="DC85" s="23"/>
     </row>
-    <row r="86" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="10" t="s">
         <v>104</v>
       </c>
@@ -17407,7 +17411,7 @@
         <v>2968</v>
       </c>
     </row>
-    <row r="87" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="10" t="s">
         <v>104</v>
       </c>
@@ -17570,7 +17574,7 @@
       <c r="DB87" s="23"/>
       <c r="DC87" s="23"/>
     </row>
-    <row r="88" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="10" t="s">
         <v>104</v>
       </c>
@@ -17737,7 +17741,7 @@
       <c r="DB88" s="23"/>
       <c r="DC88" s="23"/>
     </row>
-    <row r="89" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="10" t="s">
         <v>104</v>
       </c>
@@ -17896,7 +17900,7 @@
       <c r="DB89" s="23"/>
       <c r="DC89" s="23"/>
     </row>
-    <row r="90" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="10" t="s">
         <v>104</v>
       </c>
@@ -18059,7 +18063,7 @@
       <c r="DB90" s="23"/>
       <c r="DC90" s="23"/>
     </row>
-    <row r="91" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="10" t="s">
         <v>104</v>
       </c>
@@ -18222,7 +18226,7 @@
       <c r="DB91" s="23"/>
       <c r="DC91" s="23"/>
     </row>
-    <row r="92" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="10" t="s">
         <v>104</v>
       </c>
@@ -18389,7 +18393,7 @@
       <c r="DB92" s="23"/>
       <c r="DC92" s="23"/>
     </row>
-    <row r="93" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="10" t="s">
         <v>104</v>
       </c>
@@ -18733,7 +18737,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="95" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="10" t="s">
         <v>113</v>
       </c>
@@ -18900,7 +18904,7 @@
       <c r="DB95" s="23"/>
       <c r="DC95" s="23"/>
     </row>
-    <row r="96" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="10" t="s">
         <v>113</v>
       </c>
@@ -19067,7 +19071,7 @@
       <c r="DB96" s="23"/>
       <c r="DC96" s="23"/>
     </row>
-    <row r="97" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="10" t="s">
         <v>113</v>
       </c>
@@ -19226,7 +19230,7 @@
       <c r="DB97" s="23"/>
       <c r="DC97" s="23"/>
     </row>
-    <row r="98" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="10" t="s">
         <v>113</v>
       </c>
@@ -19395,7 +19399,7 @@
       <c r="DB98" s="23"/>
       <c r="DC98" s="23"/>
     </row>
-    <row r="99" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" s="10" t="s">
         <v>113</v>
       </c>
@@ -19560,7 +19564,7 @@
       <c r="DB99" s="23"/>
       <c r="DC99" s="23"/>
     </row>
-    <row r="100" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" s="10" t="s">
         <v>113</v>
       </c>
@@ -19751,7 +19755,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="101" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="10" t="s">
         <v>113</v>
       </c>
@@ -19912,7 +19916,7 @@
       <c r="DB101" s="23"/>
       <c r="DC101" s="23"/>
     </row>
-    <row r="102" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="10" t="s">
         <v>113</v>
       </c>
@@ -20077,7 +20081,7 @@
       <c r="DB102" s="23"/>
       <c r="DC102" s="23"/>
     </row>
-    <row r="103" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="10" t="s">
         <v>113</v>
       </c>
@@ -20260,7 +20264,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="104" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="10" t="s">
         <v>114</v>
       </c>
@@ -20425,7 +20429,7 @@
       <c r="DB104" s="23"/>
       <c r="DC104" s="23"/>
     </row>
-    <row r="105" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="10" t="s">
         <v>114</v>
       </c>
@@ -20590,7 +20594,7 @@
       <c r="DB105" s="23"/>
       <c r="DC105" s="23"/>
     </row>
-    <row r="106" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="10" t="s">
         <v>114</v>
       </c>
@@ -20751,7 +20755,7 @@
       <c r="DB106" s="23"/>
       <c r="DC106" s="23"/>
     </row>
-    <row r="107" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" s="10" t="s">
         <v>114</v>
       </c>
@@ -20942,7 +20946,7 @@
         <v>1704</v>
       </c>
     </row>
-    <row r="108" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="10" t="s">
         <v>114</v>
       </c>
@@ -21101,7 +21105,7 @@
       <c r="DB108" s="23"/>
       <c r="DC108" s="23"/>
     </row>
-    <row r="109" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" s="10" t="s">
         <v>114</v>
       </c>
@@ -21264,7 +21268,7 @@
       <c r="DB109" s="23"/>
       <c r="DC109" s="23"/>
     </row>
-    <row r="110" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="10" t="s">
         <v>120</v>
       </c>
@@ -21435,7 +21439,7 @@
       <c r="DB110" s="23"/>
       <c r="DC110" s="23"/>
     </row>
-    <row r="111" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="10" t="s">
         <v>120</v>
       </c>
@@ -21616,7 +21620,7 @@
       </c>
       <c r="DC111" s="23"/>
     </row>
-    <row r="112" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="10" t="s">
         <v>120</v>
       </c>
@@ -21801,7 +21805,7 @@
       </c>
       <c r="DC112" s="23"/>
     </row>
-    <row r="113" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="10" t="s">
         <v>120</v>
       </c>
@@ -21990,7 +21994,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="10" t="s">
         <v>120</v>
       </c>
@@ -22177,7 +22181,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="115" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="10" t="s">
         <v>120</v>
       </c>
@@ -22370,7 +22374,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="116" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="10" t="s">
         <v>290</v>
       </c>
@@ -22559,7 +22563,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="117" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="10" t="s">
         <v>290</v>
       </c>
@@ -22744,7 +22748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="10" t="s">
         <v>104</v>
       </c>
@@ -22937,7 +22941,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="10" t="s">
         <v>104</v>
       </c>
@@ -23126,7 +23130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" s="10" t="s">
         <v>104</v>
       </c>
@@ -23315,7 +23319,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="10" t="s">
         <v>104</v>
       </c>
@@ -23508,7 +23512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="10" t="s">
         <v>104</v>
       </c>
@@ -23699,7 +23703,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="123" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" s="10" t="s">
         <v>104</v>
       </c>
@@ -23890,7 +23894,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="124" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="10" t="s">
         <v>104</v>
       </c>
@@ -24085,7 +24089,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="125" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="10" t="s">
         <v>104</v>
       </c>
@@ -24272,7 +24276,7 @@
       </c>
       <c r="DC125" s="23"/>
     </row>
-    <row r="126" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" s="10" t="s">
         <v>104</v>
       </c>
@@ -24451,7 +24455,7 @@
       <c r="DB126" s="23"/>
       <c r="DC126" s="23"/>
     </row>
-    <row r="127" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="10" t="s">
         <v>104</v>
       </c>
@@ -24620,7 +24624,7 @@
       <c r="DB127" s="23"/>
       <c r="DC127" s="23"/>
     </row>
-    <row r="128" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" s="10" t="s">
         <v>104</v>
       </c>
@@ -24809,7 +24813,7 @@
       </c>
       <c r="DC128" s="23"/>
     </row>
-    <row r="129" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="10" t="s">
         <v>104</v>
       </c>
@@ -24994,7 +24998,7 @@
       </c>
       <c r="DC129" s="23"/>
     </row>
-    <row r="130" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="10" t="s">
         <v>104</v>
       </c>
@@ -25159,7 +25163,7 @@
       <c r="DB130" s="23"/>
       <c r="DC130" s="23"/>
     </row>
-    <row r="131" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="10" t="s">
         <v>104</v>
       </c>
@@ -25324,7 +25328,7 @@
       <c r="DB131" s="23"/>
       <c r="DC131" s="23"/>
     </row>
-    <row r="132" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" s="10" t="s">
         <v>104</v>
       </c>
@@ -25489,7 +25493,7 @@
       <c r="DB132" s="23"/>
       <c r="DC132" s="23"/>
     </row>
-    <row r="133" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="10" t="s">
         <v>104</v>
       </c>
@@ -25676,7 +25680,7 @@
       </c>
       <c r="DC133" s="23"/>
     </row>
-    <row r="134" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="10" t="s">
         <v>104</v>
       </c>
@@ -25859,7 +25863,7 @@
       <c r="DB134" s="23"/>
       <c r="DC134" s="23"/>
     </row>
-    <row r="135" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="10" t="s">
         <v>104</v>
       </c>
@@ -26024,7 +26028,7 @@
       <c r="DB135" s="23"/>
       <c r="DC135" s="23"/>
     </row>
-    <row r="136" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" s="10" t="s">
         <v>104</v>
       </c>
@@ -26187,7 +26191,7 @@
       <c r="DB136" s="23"/>
       <c r="DC136" s="23"/>
     </row>
-    <row r="137" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="10" t="s">
         <v>104</v>
       </c>
@@ -26374,7 +26378,7 @@
       </c>
       <c r="DC137" s="23"/>
     </row>
-    <row r="138" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="10" t="s">
         <v>104</v>
       </c>
@@ -26555,7 +26559,7 @@
       <c r="DB138" s="23"/>
       <c r="DC138" s="23"/>
     </row>
-    <row r="139" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="10" t="s">
         <v>104</v>
       </c>
@@ -26720,7 +26724,7 @@
       <c r="DB139" s="23"/>
       <c r="DC139" s="23"/>
     </row>
-    <row r="140" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="10" t="s">
         <v>104</v>
       </c>
@@ -26881,7 +26885,7 @@
       <c r="DB140" s="23"/>
       <c r="DC140" s="23"/>
     </row>
-    <row r="141" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" s="10" t="s">
         <v>104</v>
       </c>
@@ -27068,7 +27072,7 @@
       </c>
       <c r="DC141" s="23"/>
     </row>
-    <row r="142" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="10" t="s">
         <v>104</v>
       </c>
@@ -27251,7 +27255,7 @@
       <c r="DB142" s="23"/>
       <c r="DC142" s="23"/>
     </row>
-    <row r="143" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="10" t="s">
         <v>104</v>
       </c>
@@ -27416,7 +27420,7 @@
       <c r="DB143" s="23"/>
       <c r="DC143" s="23"/>
     </row>
-    <row r="144" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="10" t="s">
         <v>104</v>
       </c>
@@ -27577,7 +27581,7 @@
       <c r="DB144" s="23"/>
       <c r="DC144" s="23"/>
     </row>
-    <row r="145" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="10" t="s">
         <v>104</v>
       </c>
@@ -27760,7 +27764,7 @@
       </c>
       <c r="DC145" s="23"/>
     </row>
-    <row r="146" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="10" t="s">
         <v>104</v>
       </c>
@@ -27939,7 +27943,7 @@
       <c r="DB146" s="23"/>
       <c r="DC146" s="23"/>
     </row>
-    <row r="147" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="10" t="s">
         <v>104</v>
       </c>
@@ -28104,7 +28108,7 @@
       <c r="DB147" s="23"/>
       <c r="DC147" s="23"/>
     </row>
-    <row r="148" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="10" t="s">
         <v>104</v>
       </c>
@@ -28265,7 +28269,7 @@
       <c r="DB148" s="23"/>
       <c r="DC148" s="23"/>
     </row>
-    <row r="149" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" s="10" t="s">
         <v>104</v>
       </c>
@@ -28428,7 +28432,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="150" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" s="10" t="s">
         <v>104</v>
       </c>
@@ -28591,7 +28595,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="151" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A151" s="10" t="s">
         <v>104</v>
       </c>
@@ -28754,7 +28758,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="152" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A152" s="10" t="s">
         <v>104</v>
       </c>
@@ -28919,7 +28923,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="153" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A153" s="10" t="s">
         <v>104</v>
       </c>
@@ -29080,7 +29084,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="154" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A154" s="10" t="s">
         <v>104</v>
       </c>
@@ -29247,7 +29251,7 @@
         <v>2194</v>
       </c>
     </row>
-    <row r="155" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" s="10" t="s">
         <v>104</v>
       </c>
@@ -29585,7 +29589,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="157" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A157" s="10" t="s">
         <v>141</v>
       </c>
@@ -29756,7 +29760,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="158" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" s="10" t="s">
         <v>141</v>
       </c>
@@ -29927,7 +29931,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="159" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" s="10" t="s">
         <v>141</v>
       </c>
@@ -30118,7 +30122,7 @@
         <v>27600</v>
       </c>
     </row>
-    <row r="160" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="10" t="s">
         <v>141</v>
       </c>
@@ -30281,7 +30285,7 @@
       <c r="DB160" s="23"/>
       <c r="DC160" s="23"/>
     </row>
-    <row r="161" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" s="10" t="s">
         <v>141</v>
       </c>
@@ -30474,7 +30478,7 @@
         <v>2968</v>
       </c>
     </row>
-    <row r="162" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="10" t="s">
         <v>141</v>
       </c>
@@ -30639,7 +30643,7 @@
       <c r="DB162" s="23"/>
       <c r="DC162" s="23"/>
     </row>
-    <row r="163" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="10" t="s">
         <v>141</v>
       </c>
@@ -30808,7 +30812,7 @@
       <c r="DB163" s="23"/>
       <c r="DC163" s="23"/>
     </row>
-    <row r="164" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="10" t="s">
         <v>141</v>
       </c>
@@ -30973,7 +30977,7 @@
       <c r="DB164" s="23"/>
       <c r="DC164" s="23"/>
     </row>
-    <row r="165" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="10" t="s">
         <v>141</v>
       </c>
@@ -31142,7 +31146,7 @@
       <c r="DB165" s="23"/>
       <c r="DC165" s="23"/>
     </row>
-    <row r="166" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" s="10" t="s">
         <v>141</v>
       </c>
@@ -31307,7 +31311,7 @@
       <c r="DB166" s="23"/>
       <c r="DC166" s="23"/>
     </row>
-    <row r="167" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" s="10" t="s">
         <v>141</v>
       </c>
@@ -31490,7 +31494,7 @@
       <c r="DB167" s="23"/>
       <c r="DC167" s="23"/>
     </row>
-    <row r="168" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" s="10" t="s">
         <v>141</v>
       </c>
@@ -31657,7 +31661,7 @@
       <c r="DB168" s="23"/>
       <c r="DC168" s="23"/>
     </row>
-    <row r="169" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" s="10" t="s">
         <v>141</v>
       </c>
@@ -31818,7 +31822,7 @@
       <c r="DB169" s="23"/>
       <c r="DC169" s="23"/>
     </row>
-    <row r="170" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" s="10" t="s">
         <v>141</v>
       </c>
@@ -31999,7 +32003,7 @@
       </c>
       <c r="DC170" s="23"/>
     </row>
-    <row r="171" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" s="10" t="s">
         <v>141</v>
       </c>
@@ -32176,7 +32180,7 @@
       <c r="DB171" s="23"/>
       <c r="DC171" s="23"/>
     </row>
-    <row r="172" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" s="10" t="s">
         <v>141</v>
       </c>
@@ -32343,7 +32347,7 @@
       <c r="DB172" s="23"/>
       <c r="DC172" s="23"/>
     </row>
-    <row r="173" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A173" s="10" t="s">
         <v>141</v>
       </c>
@@ -32506,7 +32510,7 @@
       <c r="DB173" s="23"/>
       <c r="DC173" s="23"/>
     </row>
-    <row r="174" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A174" s="10" t="s">
         <v>141</v>
       </c>
@@ -32669,7 +32673,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="175" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" s="10" t="s">
         <v>141</v>
       </c>
@@ -32832,7 +32836,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="176" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" s="10" t="s">
         <v>141</v>
       </c>
@@ -32997,7 +33001,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" s="10" t="s">
         <v>141</v>
       </c>
@@ -33162,7 +33166,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="178" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" s="10" t="s">
         <v>141</v>
       </c>
@@ -33325,7 +33329,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="179" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" s="10" t="s">
         <v>141</v>
       </c>
@@ -33496,7 +33500,7 @@
         <v>2194</v>
       </c>
     </row>
-    <row r="180" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" s="10" t="s">
         <v>141</v>
       </c>
@@ -33667,7 +33671,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="181" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" s="10" t="s">
         <v>141</v>
       </c>
@@ -33838,7 +33842,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="182" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" s="10" t="s">
         <v>141</v>
       </c>
@@ -34009,7 +34013,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="183" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" s="10" t="s">
         <v>141</v>
       </c>
@@ -34180,7 +34184,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="184" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" s="10" t="s">
         <v>141</v>
       </c>
@@ -34371,7 +34375,7 @@
         <v>27600</v>
       </c>
     </row>
-    <row r="185" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" s="10" t="s">
         <v>141</v>
       </c>
@@ -34532,7 +34536,7 @@
       <c r="DB185" s="23"/>
       <c r="DC185" s="23"/>
     </row>
-    <row r="186" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" s="10" t="s">
         <v>141</v>
       </c>
@@ -34725,7 +34729,7 @@
         <v>2968</v>
       </c>
     </row>
-    <row r="187" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" s="10" t="s">
         <v>141</v>
       </c>
@@ -34892,7 +34896,7 @@
       <c r="DB187" s="23"/>
       <c r="DC187" s="23"/>
     </row>
-    <row r="188" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" s="10" t="s">
         <v>141</v>
       </c>
@@ -35061,7 +35065,7 @@
       <c r="DB188" s="23"/>
       <c r="DC188" s="23"/>
     </row>
-    <row r="189" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" s="10" t="s">
         <v>141</v>
       </c>
@@ -35224,7 +35228,7 @@
       <c r="DB189" s="23"/>
       <c r="DC189" s="23"/>
     </row>
-    <row r="190" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="10" t="s">
         <v>141</v>
       </c>
@@ -35391,7 +35395,7 @@
       <c r="DB190" s="23"/>
       <c r="DC190" s="23"/>
     </row>
-    <row r="191" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" s="10" t="s">
         <v>141</v>
       </c>
@@ -35556,7 +35560,7 @@
       <c r="DB191" s="23"/>
       <c r="DC191" s="23"/>
     </row>
-    <row r="192" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" s="10" t="s">
         <v>141</v>
       </c>
@@ -35725,7 +35729,7 @@
       <c r="DB192" s="23"/>
       <c r="DC192" s="23"/>
     </row>
-    <row r="193" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" s="10" t="s">
         <v>141</v>
       </c>
@@ -35894,7 +35898,7 @@
       <c r="DB193" s="23"/>
       <c r="DC193" s="23"/>
     </row>
-    <row r="194" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" s="10" t="s">
         <v>141</v>
       </c>
@@ -36079,7 +36083,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="195" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" s="10" t="s">
         <v>141</v>
       </c>
@@ -36250,7 +36254,7 @@
       <c r="DB195" s="23"/>
       <c r="DC195" s="23"/>
     </row>
-    <row r="196" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A196" s="10" t="s">
         <v>141</v>
       </c>
@@ -36419,7 +36423,7 @@
       <c r="DB196" s="23"/>
       <c r="DC196" s="23"/>
     </row>
-    <row r="197" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="10" t="s">
         <v>141</v>
       </c>
@@ -36580,7 +36584,7 @@
       <c r="DB197" s="23"/>
       <c r="DC197" s="23"/>
     </row>
-    <row r="198" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" s="10" t="s">
         <v>141</v>
       </c>
@@ -36751,7 +36755,7 @@
       <c r="DB198" s="23"/>
       <c r="DC198" s="23"/>
     </row>
-    <row r="199" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" s="10" t="s">
         <v>141</v>
       </c>
@@ -36918,7 +36922,7 @@
       <c r="DB199" s="23"/>
       <c r="DC199" s="23"/>
     </row>
-    <row r="200" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" s="10" t="s">
         <v>141</v>
       </c>
@@ -37109,7 +37113,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="201" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A201" s="10" t="s">
         <v>141</v>
       </c>
@@ -37270,7 +37274,7 @@
       <c r="DB201" s="23"/>
       <c r="DC201" s="23"/>
     </row>
-    <row r="202" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" s="10" t="s">
         <v>141</v>
       </c>
@@ -37435,7 +37439,7 @@
       <c r="DB202" s="23"/>
       <c r="DC202" s="23"/>
     </row>
-    <row r="203" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" s="10" t="s">
         <v>141</v>
       </c>
@@ -37618,7 +37622,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="204" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A204" s="10" t="s">
         <v>141</v>
       </c>
@@ -37783,7 +37787,7 @@
       <c r="DB204" s="23"/>
       <c r="DC204" s="23"/>
     </row>
-    <row r="205" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A205" s="10" t="s">
         <v>141</v>
       </c>
@@ -37950,7 +37954,7 @@
       <c r="DB205" s="23"/>
       <c r="DC205" s="23"/>
     </row>
-    <row r="206" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A206" s="10" t="s">
         <v>141</v>
       </c>
@@ -38113,7 +38117,7 @@
       <c r="DB206" s="23"/>
       <c r="DC206" s="23"/>
     </row>
-    <row r="207" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A207" s="10" t="s">
         <v>141</v>
       </c>
@@ -38304,7 +38308,7 @@
         <v>1704</v>
       </c>
     </row>
-    <row r="208" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A208" s="10" t="s">
         <v>141</v>
       </c>
@@ -38467,7 +38471,7 @@
       <c r="DB208" s="23"/>
       <c r="DC208" s="23"/>
     </row>
-    <row r="209" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" s="10" t="s">
         <v>141</v>
       </c>
@@ -38634,7 +38638,7 @@
       <c r="DB209" s="23"/>
       <c r="DC209" s="23"/>
     </row>
-    <row r="210" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" s="10" t="s">
         <v>141</v>
       </c>
@@ -38803,7 +38807,7 @@
       <c r="DB210" s="23"/>
       <c r="DC210" s="23"/>
     </row>
-    <row r="211" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" s="10" t="s">
         <v>141</v>
       </c>
@@ -38984,7 +38988,7 @@
       </c>
       <c r="DC211" s="23"/>
     </row>
-    <row r="212" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" s="10" t="s">
         <v>141</v>
       </c>
@@ -39169,7 +39173,7 @@
       </c>
       <c r="DC212" s="23"/>
     </row>
-    <row r="213" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" s="10" t="s">
         <v>141</v>
       </c>
@@ -39360,7 +39364,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="214" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="10" t="s">
         <v>141</v>
       </c>
@@ -39549,7 +39553,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="215" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="10" t="s">
         <v>141</v>
       </c>
@@ -39740,7 +39744,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="216" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" s="10" t="s">
         <v>141</v>
       </c>
@@ -39929,7 +39933,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="217" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" s="10" t="s">
         <v>142</v>
       </c>
@@ -40118,7 +40122,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="218" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A218" s="10" t="s">
         <v>142</v>
       </c>
@@ -40311,7 +40315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="219" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A219" s="10" t="s">
         <v>142</v>
       </c>
@@ -40496,7 +40500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" s="10" t="s">
         <v>142</v>
       </c>
@@ -40683,7 +40687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="221" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" s="10" t="s">
         <v>142</v>
       </c>
@@ -40874,7 +40878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="222" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" s="10" t="s">
         <v>142</v>
       </c>
@@ -41063,7 +41067,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="223" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" s="10" t="s">
         <v>142</v>
       </c>
@@ -41254,7 +41258,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="224" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" s="10" t="s">
         <v>142</v>
       </c>
@@ -41449,7 +41453,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="225" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" s="10" t="s">
         <v>142</v>
       </c>
@@ -41634,7 +41638,7 @@
       </c>
       <c r="DC225" s="23"/>
     </row>
-    <row r="226" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" s="10" t="s">
         <v>142</v>
       </c>
@@ -41811,7 +41815,7 @@
       <c r="DB226" s="23"/>
       <c r="DC226" s="23"/>
     </row>
-    <row r="227" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" s="10" t="s">
         <v>142</v>
       </c>
@@ -41976,7 +41980,7 @@
       <c r="DB227" s="23"/>
       <c r="DC227" s="23"/>
     </row>
-    <row r="228" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" s="10" t="s">
         <v>142</v>
       </c>
@@ -42161,7 +42165,7 @@
       </c>
       <c r="DC228" s="23"/>
     </row>
-    <row r="229" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" s="10" t="s">
         <v>142</v>
       </c>
@@ -42346,7 +42350,7 @@
       </c>
       <c r="DC229" s="23"/>
     </row>
-    <row r="230" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" s="10" t="s">
         <v>142</v>
       </c>
@@ -42513,7 +42517,7 @@
       <c r="DB230" s="23"/>
       <c r="DC230" s="23"/>
     </row>
-    <row r="231" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" s="10" t="s">
         <v>142</v>
       </c>
@@ -42680,7 +42684,7 @@
       <c r="DB231" s="23"/>
       <c r="DC231" s="23"/>
     </row>
-    <row r="232" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A232" s="10" t="s">
         <v>142</v>
       </c>
@@ -42845,7 +42849,7 @@
       <c r="DB232" s="23"/>
       <c r="DC232" s="23"/>
     </row>
-    <row r="233" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" s="10" t="s">
         <v>142</v>
       </c>
@@ -43032,7 +43036,7 @@
       </c>
       <c r="DC233" s="23"/>
     </row>
-    <row r="234" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A234" s="10" t="s">
         <v>142</v>
       </c>
@@ -43215,7 +43219,7 @@
       <c r="DB234" s="23"/>
       <c r="DC234" s="23"/>
     </row>
-    <row r="235" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" s="10" t="s">
         <v>142</v>
       </c>
@@ -43380,7 +43384,7 @@
       <c r="DB235" s="23"/>
       <c r="DC235" s="23"/>
     </row>
-    <row r="236" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" s="10" t="s">
         <v>142</v>
       </c>
@@ -43541,7 +43545,7 @@
       <c r="DB236" s="23"/>
       <c r="DC236" s="23"/>
     </row>
-    <row r="237" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" s="10" t="s">
         <v>142</v>
       </c>
@@ -43726,7 +43730,7 @@
       </c>
       <c r="DC237" s="23"/>
     </row>
-    <row r="238" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A238" s="10" t="s">
         <v>142</v>
       </c>
@@ -43889,7 +43893,7 @@
       <c r="DB238" s="23"/>
       <c r="DC238" s="23"/>
     </row>
-    <row r="239" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A239" s="10" t="s">
         <v>142</v>
       </c>
@@ -44056,7 +44060,7 @@
       <c r="DB239" s="23"/>
       <c r="DC239" s="23"/>
     </row>
-    <row r="240" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" s="10" t="s">
         <v>142</v>
       </c>
@@ -44221,7 +44225,7 @@
       <c r="DB240" s="23"/>
       <c r="DC240" s="23"/>
     </row>
-    <row r="241" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" s="10" t="s">
         <v>142</v>
       </c>
@@ -44390,7 +44394,7 @@
       <c r="DB241" s="23"/>
       <c r="DC241" s="23"/>
     </row>
-    <row r="242" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" s="10" t="s">
         <v>142</v>
       </c>
@@ -44561,7 +44565,7 @@
       <c r="DB242" s="23"/>
       <c r="DC242" s="23"/>
     </row>
-    <row r="243" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" s="10" t="s">
         <v>142</v>
       </c>
@@ -44746,7 +44750,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="244" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" s="10" t="s">
         <v>142</v>
       </c>
@@ -44915,7 +44919,7 @@
       <c r="DB244" s="23"/>
       <c r="DC244" s="23"/>
     </row>
-    <row r="245" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A245" s="10" t="s">
         <v>142</v>
       </c>
@@ -45084,7 +45088,7 @@
       <c r="DB245" s="23"/>
       <c r="DC245" s="23"/>
     </row>
-    <row r="246" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" s="10" t="s">
         <v>142</v>
       </c>
@@ -45247,7 +45251,7 @@
       <c r="DB246" s="23"/>
       <c r="DC246" s="23"/>
     </row>
-    <row r="247" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A247" s="10" t="s">
         <v>142</v>
       </c>
@@ -45418,7 +45422,7 @@
       <c r="DB247" s="23"/>
       <c r="DC247" s="23"/>
     </row>
-    <row r="248" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" s="10" t="s">
         <v>142</v>
       </c>
@@ -45583,7 +45587,7 @@
       <c r="DB248" s="23"/>
       <c r="DC248" s="23"/>
     </row>
-    <row r="249" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A249" s="10" t="s">
         <v>142</v>
       </c>
@@ -45776,7 +45780,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="250" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" s="10" t="s">
         <v>142</v>
       </c>
@@ -45941,7 +45945,7 @@
       <c r="DB250" s="23"/>
       <c r="DC250" s="23"/>
     </row>
-    <row r="251" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" s="10" t="s">
         <v>142</v>
       </c>
@@ -46108,7 +46112,7 @@
       <c r="DB251" s="23"/>
       <c r="DC251" s="23"/>
     </row>
-    <row r="252" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" s="10" t="s">
         <v>142</v>
       </c>
@@ -46291,7 +46295,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="253" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" s="10" t="s">
         <v>142</v>
       </c>
@@ -46458,7 +46462,7 @@
       <c r="DB253" s="23"/>
       <c r="DC253" s="23"/>
     </row>
-    <row r="254" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" s="10" t="s">
         <v>142</v>
       </c>
@@ -46627,7 +46631,7 @@
       <c r="DB254" s="23"/>
       <c r="DC254" s="23"/>
     </row>
-    <row r="255" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" s="10" t="s">
         <v>142</v>
       </c>
@@ -46790,7 +46794,7 @@
       <c r="DB255" s="23"/>
       <c r="DC255" s="23"/>
     </row>
-    <row r="256" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" s="10" t="s">
         <v>142</v>
       </c>
@@ -46981,7 +46985,7 @@
         <v>1704</v>
       </c>
     </row>
-    <row r="257" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" s="10" t="s">
         <v>142</v>
       </c>
@@ -47142,7 +47146,7 @@
       <c r="DB257" s="23"/>
       <c r="DC257" s="23"/>
     </row>
-    <row r="258" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" s="10" t="s">
         <v>142</v>
       </c>
@@ -47311,7 +47315,7 @@
       <c r="DB258" s="23"/>
       <c r="DC258" s="23"/>
     </row>
-    <row r="259" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A259" s="10" t="s">
         <v>142</v>
       </c>
@@ -47484,7 +47488,7 @@
       <c r="DB259" s="23"/>
       <c r="DC259" s="23"/>
     </row>
-    <row r="260" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" s="10" t="s">
         <v>142</v>
       </c>
@@ -47665,7 +47669,7 @@
       </c>
       <c r="DC260" s="23"/>
     </row>
-    <row r="261" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" s="10" t="s">
         <v>114</v>
       </c>
@@ -47850,7 +47854,7 @@
       </c>
       <c r="DC261" s="23"/>
     </row>
-    <row r="262" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262" s="10" t="s">
         <v>114</v>
       </c>
@@ -48041,7 +48045,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="263" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A263" s="10" t="s">
         <v>114</v>
       </c>
@@ -48230,7 +48234,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="264" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A264" s="10" t="s">
         <v>114</v>
       </c>
@@ -48391,7 +48395,7 @@
       <c r="DB264" s="23"/>
       <c r="DC264" s="23"/>
     </row>
-    <row r="265" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A265" s="10" t="s">
         <v>114</v>
       </c>
@@ -48582,7 +48586,7 @@
         <v>1704</v>
       </c>
     </row>
-    <row r="266" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A266" s="10" t="s">
         <v>114</v>
       </c>
@@ -48773,7 +48777,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="267" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A267" s="10" t="s">
         <v>114</v>
       </c>
@@ -48962,7 +48966,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="268" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" s="10" t="s">
         <v>114</v>
       </c>
@@ -49151,7 +49155,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="269" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A269" s="10" t="s">
         <v>114</v>
       </c>
@@ -49344,7 +49348,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="270" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" s="10" t="s">
         <v>114</v>
       </c>
@@ -49529,7 +49533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A271" s="10" t="s">
         <v>114</v>
       </c>
@@ -49716,7 +49720,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="272" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A272" s="10" t="s">
         <v>114</v>
       </c>
@@ -49907,7 +49911,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="273" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A273" s="10" t="s">
         <v>114</v>
       </c>
@@ -50096,7 +50100,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="274" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A274" s="10" t="s">
         <v>114</v>
       </c>
@@ -50287,7 +50291,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="275" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A275" s="10" t="s">
         <v>114</v>
       </c>
@@ -50482,7 +50486,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="276" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A276" s="10" t="s">
         <v>114</v>
       </c>
@@ -50667,7 +50671,7 @@
       </c>
       <c r="DC276" s="23"/>
     </row>
-    <row r="277" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A277" s="10" t="s">
         <v>114</v>
       </c>
@@ -50844,7 +50848,7 @@
       <c r="DB277" s="23"/>
       <c r="DC277" s="23"/>
     </row>
-    <row r="278" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A278" s="10" t="s">
         <v>114</v>
       </c>
@@ -51009,7 +51013,7 @@
       <c r="DB278" s="23"/>
       <c r="DC278" s="23"/>
     </row>
-    <row r="279" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A279" s="10" t="s">
         <v>114</v>
       </c>
@@ -51194,7 +51198,7 @@
       </c>
       <c r="DC279" s="23"/>
     </row>
-    <row r="280" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A280" s="10" t="s">
         <v>114</v>
       </c>
@@ -51379,7 +51383,7 @@
       </c>
       <c r="DC280" s="23"/>
     </row>
-    <row r="281" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A281" s="10" t="s">
         <v>114</v>
       </c>
@@ -51546,7 +51550,7 @@
       <c r="DB281" s="23"/>
       <c r="DC281" s="23"/>
     </row>
-    <row r="282" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A282" s="10" t="s">
         <v>114</v>
       </c>
@@ -51713,7 +51717,7 @@
       <c r="DB282" s="23"/>
       <c r="DC282" s="23"/>
     </row>
-    <row r="283" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A283" s="10" t="s">
         <v>114</v>
       </c>
@@ -51878,7 +51882,7 @@
       <c r="DB283" s="23"/>
       <c r="DC283" s="23"/>
     </row>
-    <row r="284" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A284" s="10" t="s">
         <v>114</v>
       </c>
@@ -52065,7 +52069,7 @@
       </c>
       <c r="DC284" s="23"/>
     </row>
-    <row r="285" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A285" s="10" t="s">
         <v>114</v>
       </c>
@@ -52248,7 +52252,7 @@
       <c r="DB285" s="23"/>
       <c r="DC285" s="23"/>
     </row>
-    <row r="286" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A286" s="10" t="s">
         <v>114</v>
       </c>
@@ -52413,7 +52417,7 @@
       <c r="DB286" s="23"/>
       <c r="DC286" s="23"/>
     </row>
-    <row r="287" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A287" s="10" t="s">
         <v>114</v>
       </c>
@@ -52574,7 +52578,7 @@
       <c r="DB287" s="23"/>
       <c r="DC287" s="23"/>
     </row>
-    <row r="288" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A288" s="10" t="s">
         <v>104</v>
       </c>
@@ -52759,7 +52763,7 @@
       </c>
       <c r="DC288" s="23"/>
     </row>
-    <row r="289" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A289" s="10" t="s">
         <v>104</v>
       </c>
@@ -52922,7 +52926,7 @@
       <c r="DB289" s="23"/>
       <c r="DC289" s="23"/>
     </row>
-    <row r="290" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A290" s="10" t="s">
         <v>104</v>
       </c>
@@ -53089,7 +53093,7 @@
       <c r="DB290" s="23"/>
       <c r="DC290" s="23"/>
     </row>
-    <row r="291" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A291" s="10" t="s">
         <v>104</v>
       </c>
@@ -53254,7 +53258,7 @@
       <c r="DB291" s="23"/>
       <c r="DC291" s="23"/>
     </row>
-    <row r="292" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A292" s="10" t="s">
         <v>104</v>
       </c>
@@ -53423,7 +53427,7 @@
       <c r="DB292" s="23"/>
       <c r="DC292" s="23"/>
     </row>
-    <row r="293" spans="1:107" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:107" hidden="1" x14ac:dyDescent="0.2">
       <c r="A293" s="10" t="s">
         <v>104</v>
       </c>
@@ -53595,6 +53599,23 @@
       <c r="DC293" s="23"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:DC293" xr:uid="{2B013508-E228-5F48-8A4D-5ECE74B70E01}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="JEEP"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="EEU"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="15">
+      <filters>
+        <dateGroupItem year="2026" dateTimeGrouping="year"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>